<commit_message>
producto a excel 1
</commit_message>
<xml_diff>
--- a/data/excel.xlsx
+++ b/data/excel.xlsx
@@ -1,34 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abiga\Documents\New project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BDA169E-0D56-4749-B47C-5F53A3E34BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14148AB6-FD36-460F-888C-845CCB44B34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AZUCAR" sheetId="4" r:id="rId1"/>
     <sheet name="GRANOS" sheetId="6" r:id="rId2"/>
-    <sheet name="PLASTICOS" sheetId="9" r:id="rId3"/>
-    <sheet name="MADERA" sheetId="10" r:id="rId4"/>
-    <sheet name="MATERIALES DE CONSTRUCCION" sheetId="7" r:id="rId5"/>
-    <sheet name="PRODUCTOS ELECTRONICOS" sheetId="11" r:id="rId6"/>
-    <sheet name="TELEFONOS CELULARES" sheetId="12" r:id="rId7"/>
-    <sheet name="Hoja1" sheetId="13" r:id="rId8"/>
-    <sheet name="Hoja6" sheetId="8" state="hidden" r:id="rId9"/>
+    <sheet name="Hoja2" sheetId="14" r:id="rId3"/>
+    <sheet name="PLASTICOS" sheetId="9" r:id="rId4"/>
+    <sheet name="MADERA" sheetId="10" r:id="rId5"/>
+    <sheet name="MATERIALES DE CONSTRUCCION" sheetId="7" r:id="rId6"/>
+    <sheet name="PRODUCTOS ELECTRONICOS" sheetId="11" r:id="rId7"/>
+    <sheet name="TELEFONOS CELULARES" sheetId="12" r:id="rId8"/>
+    <sheet name="22415 cod aduanero" sheetId="13" r:id="rId9"/>
+    <sheet name="Hoja6" sheetId="8" state="hidden" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1743" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1752" uniqueCount="437">
   <si>
     <t>Bolsa ingenio</t>
   </si>
@@ -1324,6 +1325,21 @@
   </si>
   <si>
     <t>nueces</t>
+  </si>
+  <si>
+    <t>PRODUCTO</t>
+  </si>
+  <si>
+    <t>HOJA DE COCA</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRAMO </t>
+  </si>
+  <si>
+    <t>CLORHIDRATO DE COCAINA</t>
   </si>
 </sst>
 </file>
@@ -1427,7 +1443,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1464,7 +1480,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2047,6 +2062,1580 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B40AC6E-5AA6-4139-9D9D-0C1E963453B3}">
+  <dimension ref="A1:E103"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2">
+        <v>12000</v>
+      </c>
+      <c r="E2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3">
+        <v>22000</v>
+      </c>
+      <c r="E3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4">
+        <v>7300</v>
+      </c>
+      <c r="E4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5">
+        <v>9000</v>
+      </c>
+      <c r="E5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6">
+        <v>14000</v>
+      </c>
+      <c r="E6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7">
+        <v>18000</v>
+      </c>
+      <c r="E7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8">
+        <v>15000</v>
+      </c>
+      <c r="E8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9">
+        <v>14000</v>
+      </c>
+      <c r="E9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10">
+        <v>20000</v>
+      </c>
+      <c r="E10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11">
+        <v>16000</v>
+      </c>
+      <c r="E11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13">
+        <v>40000</v>
+      </c>
+      <c r="E13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14">
+        <v>42000</v>
+      </c>
+      <c r="E14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" t="s">
+        <v>93</v>
+      </c>
+      <c r="C15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15">
+        <v>45000</v>
+      </c>
+      <c r="E15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16">
+        <v>135000</v>
+      </c>
+      <c r="E16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" t="s">
+        <v>95</v>
+      </c>
+      <c r="C17" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17">
+        <v>120000</v>
+      </c>
+      <c r="E17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18">
+        <v>105000</v>
+      </c>
+      <c r="E18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" t="s">
+        <v>97</v>
+      </c>
+      <c r="C19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19">
+        <v>110000</v>
+      </c>
+      <c r="E19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" t="s">
+        <v>98</v>
+      </c>
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20">
+        <v>85000</v>
+      </c>
+      <c r="E20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" t="s">
+        <v>99</v>
+      </c>
+      <c r="C21" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21">
+        <v>65000</v>
+      </c>
+      <c r="E21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>89</v>
+      </c>
+      <c r="B22" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" t="s">
+        <v>91</v>
+      </c>
+      <c r="D22">
+        <v>70000</v>
+      </c>
+      <c r="E22" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>89</v>
+      </c>
+      <c r="B23" t="s">
+        <v>101</v>
+      </c>
+      <c r="C23" t="s">
+        <v>91</v>
+      </c>
+      <c r="D23">
+        <v>60000</v>
+      </c>
+      <c r="E23" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" t="s">
+        <v>103</v>
+      </c>
+      <c r="C25" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25">
+        <v>230</v>
+      </c>
+      <c r="E25" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>102</v>
+      </c>
+      <c r="B26" t="s">
+        <v>105</v>
+      </c>
+      <c r="C26" t="s">
+        <v>104</v>
+      </c>
+      <c r="D26">
+        <v>1200</v>
+      </c>
+      <c r="E26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>102</v>
+      </c>
+      <c r="B27" t="s">
+        <v>106</v>
+      </c>
+      <c r="C27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27">
+        <v>1800</v>
+      </c>
+      <c r="E27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" t="s">
+        <v>107</v>
+      </c>
+      <c r="C28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28">
+        <v>2500</v>
+      </c>
+      <c r="E28" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" t="s">
+        <v>104</v>
+      </c>
+      <c r="D29">
+        <v>3000</v>
+      </c>
+      <c r="E29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B30" t="s">
+        <v>109</v>
+      </c>
+      <c r="C30" t="s">
+        <v>104</v>
+      </c>
+      <c r="D30">
+        <v>2100</v>
+      </c>
+      <c r="E30" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" t="s">
+        <v>110</v>
+      </c>
+      <c r="C31" t="s">
+        <v>104</v>
+      </c>
+      <c r="D31">
+        <v>2500</v>
+      </c>
+      <c r="E31" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" t="s">
+        <v>111</v>
+      </c>
+      <c r="C32" t="s">
+        <v>104</v>
+      </c>
+      <c r="D32">
+        <v>6500</v>
+      </c>
+      <c r="E32" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33">
+        <v>3500</v>
+      </c>
+      <c r="E33" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" t="s">
+        <v>113</v>
+      </c>
+      <c r="C34" t="s">
+        <v>104</v>
+      </c>
+      <c r="D34">
+        <v>3200</v>
+      </c>
+      <c r="E34" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>114</v>
+      </c>
+      <c r="B36" t="s">
+        <v>115</v>
+      </c>
+      <c r="C36" t="s">
+        <v>91</v>
+      </c>
+      <c r="D36">
+        <v>140000</v>
+      </c>
+      <c r="E36" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>114</v>
+      </c>
+      <c r="B37" t="s">
+        <v>116</v>
+      </c>
+      <c r="C37" t="s">
+        <v>91</v>
+      </c>
+      <c r="D37">
+        <v>135000</v>
+      </c>
+      <c r="E37" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>114</v>
+      </c>
+      <c r="B38" t="s">
+        <v>117</v>
+      </c>
+      <c r="C38" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38">
+        <v>145000</v>
+      </c>
+      <c r="E38" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>114</v>
+      </c>
+      <c r="B39" t="s">
+        <v>118</v>
+      </c>
+      <c r="C39" t="s">
+        <v>119</v>
+      </c>
+      <c r="D39">
+        <v>9000</v>
+      </c>
+      <c r="E39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>114</v>
+      </c>
+      <c r="B40" t="s">
+        <v>120</v>
+      </c>
+      <c r="C40" t="s">
+        <v>119</v>
+      </c>
+      <c r="D40">
+        <v>11000</v>
+      </c>
+      <c r="E40" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>114</v>
+      </c>
+      <c r="B41" t="s">
+        <v>121</v>
+      </c>
+      <c r="C41" t="s">
+        <v>104</v>
+      </c>
+      <c r="D41">
+        <v>4500</v>
+      </c>
+      <c r="E41" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>114</v>
+      </c>
+      <c r="B42" t="s">
+        <v>122</v>
+      </c>
+      <c r="C42" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42">
+        <v>4200</v>
+      </c>
+      <c r="E42" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>114</v>
+      </c>
+      <c r="B43" t="s">
+        <v>123</v>
+      </c>
+      <c r="C43" t="s">
+        <v>124</v>
+      </c>
+      <c r="D43">
+        <v>55000</v>
+      </c>
+      <c r="E43" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>125</v>
+      </c>
+      <c r="B45" t="s">
+        <v>126</v>
+      </c>
+      <c r="C45" t="s">
+        <v>127</v>
+      </c>
+      <c r="D45">
+        <v>8000</v>
+      </c>
+      <c r="E45" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>125</v>
+      </c>
+      <c r="B46" t="s">
+        <v>128</v>
+      </c>
+      <c r="C46" t="s">
+        <v>127</v>
+      </c>
+      <c r="D46">
+        <v>11000</v>
+      </c>
+      <c r="E46" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>125</v>
+      </c>
+      <c r="B47" t="s">
+        <v>129</v>
+      </c>
+      <c r="C47" t="s">
+        <v>127</v>
+      </c>
+      <c r="D47">
+        <v>15000</v>
+      </c>
+      <c r="E47" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>125</v>
+      </c>
+      <c r="B48" t="s">
+        <v>130</v>
+      </c>
+      <c r="C48" t="s">
+        <v>127</v>
+      </c>
+      <c r="D48">
+        <v>19000</v>
+      </c>
+      <c r="E48" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>125</v>
+      </c>
+      <c r="B49" t="s">
+        <v>131</v>
+      </c>
+      <c r="C49" t="s">
+        <v>127</v>
+      </c>
+      <c r="D49">
+        <v>26000</v>
+      </c>
+      <c r="E49" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>125</v>
+      </c>
+      <c r="B50" t="s">
+        <v>132</v>
+      </c>
+      <c r="C50" t="s">
+        <v>124</v>
+      </c>
+      <c r="D50">
+        <v>10000</v>
+      </c>
+      <c r="E50" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>125</v>
+      </c>
+      <c r="B51" t="s">
+        <v>133</v>
+      </c>
+      <c r="C51" t="s">
+        <v>134</v>
+      </c>
+      <c r="D51">
+        <v>1600</v>
+      </c>
+      <c r="E51" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>125</v>
+      </c>
+      <c r="B52" t="s">
+        <v>135</v>
+      </c>
+      <c r="C52" t="s">
+        <v>134</v>
+      </c>
+      <c r="D52">
+        <v>1400</v>
+      </c>
+      <c r="E52" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>125</v>
+      </c>
+      <c r="B53" t="s">
+        <v>136</v>
+      </c>
+      <c r="C53" t="s">
+        <v>134</v>
+      </c>
+      <c r="D53">
+        <v>2000</v>
+      </c>
+      <c r="E53" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>125</v>
+      </c>
+      <c r="B54" t="s">
+        <v>137</v>
+      </c>
+      <c r="C54" t="s">
+        <v>119</v>
+      </c>
+      <c r="D54">
+        <v>8500</v>
+      </c>
+      <c r="E54" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>125</v>
+      </c>
+      <c r="B55" t="s">
+        <v>138</v>
+      </c>
+      <c r="C55" t="s">
+        <v>119</v>
+      </c>
+      <c r="D55">
+        <v>9000</v>
+      </c>
+      <c r="E55" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>125</v>
+      </c>
+      <c r="B56" t="s">
+        <v>139</v>
+      </c>
+      <c r="C56" t="s">
+        <v>119</v>
+      </c>
+      <c r="D56">
+        <v>12000</v>
+      </c>
+      <c r="E56" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>140</v>
+      </c>
+      <c r="B58" t="s">
+        <v>141</v>
+      </c>
+      <c r="C58" t="s">
+        <v>124</v>
+      </c>
+      <c r="D58">
+        <v>32000</v>
+      </c>
+      <c r="E58" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>140</v>
+      </c>
+      <c r="B59" t="s">
+        <v>142</v>
+      </c>
+      <c r="C59" t="s">
+        <v>124</v>
+      </c>
+      <c r="D59">
+        <v>38000</v>
+      </c>
+      <c r="E59" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>140</v>
+      </c>
+      <c r="B60" t="s">
+        <v>143</v>
+      </c>
+      <c r="C60" t="s">
+        <v>124</v>
+      </c>
+      <c r="D60">
+        <v>45000</v>
+      </c>
+      <c r="E60" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>140</v>
+      </c>
+      <c r="B61" t="s">
+        <v>144</v>
+      </c>
+      <c r="C61" t="s">
+        <v>124</v>
+      </c>
+      <c r="D61">
+        <v>30000</v>
+      </c>
+      <c r="E61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>140</v>
+      </c>
+      <c r="B62" t="s">
+        <v>145</v>
+      </c>
+      <c r="C62" t="s">
+        <v>124</v>
+      </c>
+      <c r="D62">
+        <v>42000</v>
+      </c>
+      <c r="E62" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>146</v>
+      </c>
+      <c r="B64" t="s">
+        <v>147</v>
+      </c>
+      <c r="C64" t="s">
+        <v>119</v>
+      </c>
+      <c r="D64">
+        <v>9000</v>
+      </c>
+      <c r="E64" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>146</v>
+      </c>
+      <c r="B65" t="s">
+        <v>148</v>
+      </c>
+      <c r="C65" t="s">
+        <v>119</v>
+      </c>
+      <c r="D65">
+        <v>8000</v>
+      </c>
+      <c r="E65" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>146</v>
+      </c>
+      <c r="B66" t="s">
+        <v>149</v>
+      </c>
+      <c r="C66" t="s">
+        <v>119</v>
+      </c>
+      <c r="D66">
+        <v>8500</v>
+      </c>
+      <c r="E66" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>146</v>
+      </c>
+      <c r="B67" t="s">
+        <v>150</v>
+      </c>
+      <c r="C67" t="s">
+        <v>104</v>
+      </c>
+      <c r="D67">
+        <v>18000</v>
+      </c>
+      <c r="E67" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>146</v>
+      </c>
+      <c r="B68" t="s">
+        <v>151</v>
+      </c>
+      <c r="C68" t="s">
+        <v>124</v>
+      </c>
+      <c r="D68">
+        <v>15000</v>
+      </c>
+      <c r="E68" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>146</v>
+      </c>
+      <c r="B69" t="s">
+        <v>152</v>
+      </c>
+      <c r="C69" t="s">
+        <v>124</v>
+      </c>
+      <c r="D69">
+        <v>16000</v>
+      </c>
+      <c r="E69" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>146</v>
+      </c>
+      <c r="B70" t="s">
+        <v>153</v>
+      </c>
+      <c r="C70" t="s">
+        <v>124</v>
+      </c>
+      <c r="D70">
+        <v>20000</v>
+      </c>
+      <c r="E70" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>146</v>
+      </c>
+      <c r="B71" t="s">
+        <v>154</v>
+      </c>
+      <c r="C71" t="s">
+        <v>124</v>
+      </c>
+      <c r="D71">
+        <v>22000</v>
+      </c>
+      <c r="E71" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>155</v>
+      </c>
+      <c r="B73" t="s">
+        <v>156</v>
+      </c>
+      <c r="C73" t="s">
+        <v>124</v>
+      </c>
+      <c r="D73">
+        <v>15000</v>
+      </c>
+      <c r="E73" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>155</v>
+      </c>
+      <c r="B74" t="s">
+        <v>157</v>
+      </c>
+      <c r="C74" t="s">
+        <v>124</v>
+      </c>
+      <c r="D74">
+        <v>19000</v>
+      </c>
+      <c r="E74" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>155</v>
+      </c>
+      <c r="B75" t="s">
+        <v>158</v>
+      </c>
+      <c r="C75" t="s">
+        <v>124</v>
+      </c>
+      <c r="D75">
+        <v>12000</v>
+      </c>
+      <c r="E75" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>155</v>
+      </c>
+      <c r="B76" t="s">
+        <v>159</v>
+      </c>
+      <c r="C76" t="s">
+        <v>124</v>
+      </c>
+      <c r="D76">
+        <v>20000</v>
+      </c>
+      <c r="E76" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>155</v>
+      </c>
+      <c r="B77" t="s">
+        <v>160</v>
+      </c>
+      <c r="C77" t="s">
+        <v>161</v>
+      </c>
+      <c r="D77">
+        <v>55000</v>
+      </c>
+      <c r="E77" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>162</v>
+      </c>
+      <c r="B79" t="s">
+        <v>163</v>
+      </c>
+      <c r="C79" t="s">
+        <v>124</v>
+      </c>
+      <c r="D79">
+        <v>22000</v>
+      </c>
+      <c r="E79" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>162</v>
+      </c>
+      <c r="B80" t="s">
+        <v>164</v>
+      </c>
+      <c r="C80" t="s">
+        <v>124</v>
+      </c>
+      <c r="D80">
+        <v>45000</v>
+      </c>
+      <c r="E80" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>162</v>
+      </c>
+      <c r="B81" t="s">
+        <v>165</v>
+      </c>
+      <c r="C81" t="s">
+        <v>124</v>
+      </c>
+      <c r="D81">
+        <v>28000</v>
+      </c>
+      <c r="E81" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>162</v>
+      </c>
+      <c r="B82" t="s">
+        <v>166</v>
+      </c>
+      <c r="C82" t="s">
+        <v>124</v>
+      </c>
+      <c r="D82">
+        <v>60000</v>
+      </c>
+      <c r="E82" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>162</v>
+      </c>
+      <c r="B83" t="s">
+        <v>167</v>
+      </c>
+      <c r="C83" t="s">
+        <v>124</v>
+      </c>
+      <c r="D83">
+        <v>35000</v>
+      </c>
+      <c r="E83" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>168</v>
+      </c>
+      <c r="B85" t="s">
+        <v>169</v>
+      </c>
+      <c r="C85" t="s">
+        <v>170</v>
+      </c>
+      <c r="D85">
+        <v>90000</v>
+      </c>
+      <c r="E85" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>168</v>
+      </c>
+      <c r="B86" t="s">
+        <v>171</v>
+      </c>
+      <c r="C86" t="s">
+        <v>170</v>
+      </c>
+      <c r="D86">
+        <v>110000</v>
+      </c>
+      <c r="E86" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>168</v>
+      </c>
+      <c r="B87" t="s">
+        <v>172</v>
+      </c>
+      <c r="C87" t="s">
+        <v>173</v>
+      </c>
+      <c r="D87">
+        <v>35000</v>
+      </c>
+      <c r="E87" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>168</v>
+      </c>
+      <c r="B88" t="s">
+        <v>174</v>
+      </c>
+      <c r="C88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D88">
+        <v>30000</v>
+      </c>
+      <c r="E88" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>168</v>
+      </c>
+      <c r="B89" t="s">
+        <v>175</v>
+      </c>
+      <c r="C89" t="s">
+        <v>170</v>
+      </c>
+      <c r="D89">
+        <v>120000</v>
+      </c>
+      <c r="E89" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>176</v>
+      </c>
+      <c r="B91" t="s">
+        <v>177</v>
+      </c>
+      <c r="C91" t="s">
+        <v>119</v>
+      </c>
+      <c r="D91">
+        <v>10000</v>
+      </c>
+      <c r="E91" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>176</v>
+      </c>
+      <c r="B92" t="s">
+        <v>178</v>
+      </c>
+      <c r="C92" t="s">
+        <v>119</v>
+      </c>
+      <c r="D92">
+        <v>7000</v>
+      </c>
+      <c r="E92" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>176</v>
+      </c>
+      <c r="B93" t="s">
+        <v>179</v>
+      </c>
+      <c r="C93" t="s">
+        <v>104</v>
+      </c>
+      <c r="D93">
+        <v>2500</v>
+      </c>
+      <c r="E93" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>176</v>
+      </c>
+      <c r="B94" t="s">
+        <v>180</v>
+      </c>
+      <c r="C94" t="s">
+        <v>104</v>
+      </c>
+      <c r="D94">
+        <v>9000</v>
+      </c>
+      <c r="E94" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>176</v>
+      </c>
+      <c r="B95" t="s">
+        <v>181</v>
+      </c>
+      <c r="C95" t="s">
+        <v>104</v>
+      </c>
+      <c r="D95">
+        <v>55000</v>
+      </c>
+      <c r="E95" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>182</v>
+      </c>
+      <c r="B97" t="s">
+        <v>183</v>
+      </c>
+      <c r="C97" t="s">
+        <v>119</v>
+      </c>
+      <c r="D97">
+        <v>1200</v>
+      </c>
+      <c r="E97" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>182</v>
+      </c>
+      <c r="B98" t="s">
+        <v>184</v>
+      </c>
+      <c r="C98" t="s">
+        <v>119</v>
+      </c>
+      <c r="D98">
+        <v>1700</v>
+      </c>
+      <c r="E98" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>182</v>
+      </c>
+      <c r="B99" t="s">
+        <v>185</v>
+      </c>
+      <c r="C99" t="s">
+        <v>119</v>
+      </c>
+      <c r="D99">
+        <v>800</v>
+      </c>
+      <c r="E99" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>182</v>
+      </c>
+      <c r="B100" t="s">
+        <v>186</v>
+      </c>
+      <c r="C100" t="s">
+        <v>104</v>
+      </c>
+      <c r="D100">
+        <v>2000</v>
+      </c>
+      <c r="E100" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>182</v>
+      </c>
+      <c r="B101" t="s">
+        <v>187</v>
+      </c>
+      <c r="C101" t="s">
+        <v>104</v>
+      </c>
+      <c r="D101">
+        <v>35000</v>
+      </c>
+      <c r="E101" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>182</v>
+      </c>
+      <c r="B102" t="s">
+        <v>188</v>
+      </c>
+      <c r="C102" t="s">
+        <v>104</v>
+      </c>
+      <c r="D102">
+        <v>3500</v>
+      </c>
+      <c r="E102" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>182</v>
+      </c>
+      <c r="B103" t="s">
+        <v>189</v>
+      </c>
+      <c r="C103" t="s">
+        <v>104</v>
+      </c>
+      <c r="D103">
+        <v>3200</v>
+      </c>
+      <c r="E103" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0756568B-799C-4417-9FD5-CA21567FA36E}">
   <dimension ref="A1:H22"/>
@@ -2339,7 +3928,7 @@
       <c r="F14" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H14" s="18"/>
+      <c r="H14" s="17"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
@@ -2482,7 +4071,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="8" t="s">
         <v>35</v>
       </c>
       <c r="B22" s="4" t="s">
@@ -2497,7 +4086,7 @@
       <c r="E22" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="16" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2520,6 +4109,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15575E2F-B7E9-4EB5-A791-7D7E5CF1065C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE5B732E-FF65-48B2-A0B0-FFF7B3B5DD44}">
   <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3454,7 +5052,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4933F15-821D-43F0-B734-73373F78EC52}">
   <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4745,7 +6343,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2ED5D93-0BF9-4D0B-A000-F761D38B7B46}">
   <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6333,7 +7931,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E658A0D8-3AAB-48EF-8FBD-2662AC5F929D}">
   <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7255,7 +8853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D8FF1F2-8F62-4B32-A230-1AEFCB8D93C5}">
   <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7884,1582 +9482,55 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{748F122F-7CC3-499F-98B9-01D3B28FD4BC}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B40AC6E-5AA6-4139-9D9D-0C1E963453B3}">
-  <dimension ref="A1:E103"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="33.7109375" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="10" t="s">
+        <v>432</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="E1" t="s">
-        <v>34</v>
+      <c r="E1" s="10" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>74</v>
-      </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>433</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>434</v>
       </c>
       <c r="D2">
-        <v>12000</v>
-      </c>
-      <c r="E2" t="s">
-        <v>77</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>74</v>
-      </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>436</v>
       </c>
       <c r="C3" t="s">
-        <v>79</v>
+        <v>435</v>
       </c>
       <c r="D3">
-        <v>22000</v>
-      </c>
-      <c r="E3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D4">
-        <v>7300</v>
-      </c>
-      <c r="E4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5">
-        <v>9000</v>
-      </c>
-      <c r="E5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C6" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6">
         <v>14000</v>
-      </c>
-      <c r="E6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" t="s">
-        <v>79</v>
-      </c>
-      <c r="D7">
-        <v>18000</v>
-      </c>
-      <c r="E7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8">
-        <v>15000</v>
-      </c>
-      <c r="E8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" t="s">
-        <v>86</v>
-      </c>
-      <c r="C9" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9">
-        <v>14000</v>
-      </c>
-      <c r="E9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B10" t="s">
-        <v>87</v>
-      </c>
-      <c r="C10" t="s">
-        <v>79</v>
-      </c>
-      <c r="D10">
-        <v>20000</v>
-      </c>
-      <c r="E10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" t="s">
-        <v>79</v>
-      </c>
-      <c r="D11">
-        <v>16000</v>
-      </c>
-      <c r="E11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>89</v>
-      </c>
-      <c r="B13" t="s">
-        <v>90</v>
-      </c>
-      <c r="C13" t="s">
-        <v>91</v>
-      </c>
-      <c r="D13">
-        <v>40000</v>
-      </c>
-      <c r="E13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>89</v>
-      </c>
-      <c r="B14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D14">
-        <v>42000</v>
-      </c>
-      <c r="E14" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" t="s">
-        <v>93</v>
-      </c>
-      <c r="C15" t="s">
-        <v>91</v>
-      </c>
-      <c r="D15">
-        <v>45000</v>
-      </c>
-      <c r="E15" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" t="s">
-        <v>94</v>
-      </c>
-      <c r="C16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D16">
-        <v>135000</v>
-      </c>
-      <c r="E16" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" t="s">
-        <v>95</v>
-      </c>
-      <c r="C17" t="s">
-        <v>91</v>
-      </c>
-      <c r="D17">
-        <v>120000</v>
-      </c>
-      <c r="E17" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>89</v>
-      </c>
-      <c r="B18" t="s">
-        <v>96</v>
-      </c>
-      <c r="C18" t="s">
-        <v>91</v>
-      </c>
-      <c r="D18">
-        <v>105000</v>
-      </c>
-      <c r="E18" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>89</v>
-      </c>
-      <c r="B19" t="s">
-        <v>97</v>
-      </c>
-      <c r="C19" t="s">
-        <v>91</v>
-      </c>
-      <c r="D19">
-        <v>110000</v>
-      </c>
-      <c r="E19" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>89</v>
-      </c>
-      <c r="B20" t="s">
-        <v>98</v>
-      </c>
-      <c r="C20" t="s">
-        <v>91</v>
-      </c>
-      <c r="D20">
-        <v>85000</v>
-      </c>
-      <c r="E20" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>89</v>
-      </c>
-      <c r="B21" t="s">
-        <v>99</v>
-      </c>
-      <c r="C21" t="s">
-        <v>91</v>
-      </c>
-      <c r="D21">
-        <v>65000</v>
-      </c>
-      <c r="E21" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B22" t="s">
-        <v>100</v>
-      </c>
-      <c r="C22" t="s">
-        <v>91</v>
-      </c>
-      <c r="D22">
-        <v>70000</v>
-      </c>
-      <c r="E22" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>89</v>
-      </c>
-      <c r="B23" t="s">
-        <v>101</v>
-      </c>
-      <c r="C23" t="s">
-        <v>91</v>
-      </c>
-      <c r="D23">
-        <v>60000</v>
-      </c>
-      <c r="E23" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>102</v>
-      </c>
-      <c r="B25" t="s">
-        <v>103</v>
-      </c>
-      <c r="C25" t="s">
-        <v>104</v>
-      </c>
-      <c r="D25">
-        <v>230</v>
-      </c>
-      <c r="E25" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>102</v>
-      </c>
-      <c r="B26" t="s">
-        <v>105</v>
-      </c>
-      <c r="C26" t="s">
-        <v>104</v>
-      </c>
-      <c r="D26">
-        <v>1200</v>
-      </c>
-      <c r="E26" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>102</v>
-      </c>
-      <c r="B27" t="s">
-        <v>106</v>
-      </c>
-      <c r="C27" t="s">
-        <v>104</v>
-      </c>
-      <c r="D27">
-        <v>1800</v>
-      </c>
-      <c r="E27" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>102</v>
-      </c>
-      <c r="B28" t="s">
-        <v>107</v>
-      </c>
-      <c r="C28" t="s">
-        <v>104</v>
-      </c>
-      <c r="D28">
-        <v>2500</v>
-      </c>
-      <c r="E28" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>102</v>
-      </c>
-      <c r="B29" t="s">
-        <v>108</v>
-      </c>
-      <c r="C29" t="s">
-        <v>104</v>
-      </c>
-      <c r="D29">
-        <v>3000</v>
-      </c>
-      <c r="E29" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>102</v>
-      </c>
-      <c r="B30" t="s">
-        <v>109</v>
-      </c>
-      <c r="C30" t="s">
-        <v>104</v>
-      </c>
-      <c r="D30">
-        <v>2100</v>
-      </c>
-      <c r="E30" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>102</v>
-      </c>
-      <c r="B31" t="s">
-        <v>110</v>
-      </c>
-      <c r="C31" t="s">
-        <v>104</v>
-      </c>
-      <c r="D31">
-        <v>2500</v>
-      </c>
-      <c r="E31" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>102</v>
-      </c>
-      <c r="B32" t="s">
-        <v>111</v>
-      </c>
-      <c r="C32" t="s">
-        <v>104</v>
-      </c>
-      <c r="D32">
-        <v>6500</v>
-      </c>
-      <c r="E32" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>102</v>
-      </c>
-      <c r="B33" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" t="s">
-        <v>104</v>
-      </c>
-      <c r="D33">
-        <v>3500</v>
-      </c>
-      <c r="E33" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>102</v>
-      </c>
-      <c r="B34" t="s">
-        <v>113</v>
-      </c>
-      <c r="C34" t="s">
-        <v>104</v>
-      </c>
-      <c r="D34">
-        <v>3200</v>
-      </c>
-      <c r="E34" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>114</v>
-      </c>
-      <c r="B36" t="s">
-        <v>115</v>
-      </c>
-      <c r="C36" t="s">
-        <v>91</v>
-      </c>
-      <c r="D36">
-        <v>140000</v>
-      </c>
-      <c r="E36" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>114</v>
-      </c>
-      <c r="B37" t="s">
-        <v>116</v>
-      </c>
-      <c r="C37" t="s">
-        <v>91</v>
-      </c>
-      <c r="D37">
-        <v>135000</v>
-      </c>
-      <c r="E37" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>114</v>
-      </c>
-      <c r="B38" t="s">
-        <v>117</v>
-      </c>
-      <c r="C38" t="s">
-        <v>91</v>
-      </c>
-      <c r="D38">
-        <v>145000</v>
-      </c>
-      <c r="E38" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>114</v>
-      </c>
-      <c r="B39" t="s">
-        <v>118</v>
-      </c>
-      <c r="C39" t="s">
-        <v>119</v>
-      </c>
-      <c r="D39">
-        <v>9000</v>
-      </c>
-      <c r="E39" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>114</v>
-      </c>
-      <c r="B40" t="s">
-        <v>120</v>
-      </c>
-      <c r="C40" t="s">
-        <v>119</v>
-      </c>
-      <c r="D40">
-        <v>11000</v>
-      </c>
-      <c r="E40" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>114</v>
-      </c>
-      <c r="B41" t="s">
-        <v>121</v>
-      </c>
-      <c r="C41" t="s">
-        <v>104</v>
-      </c>
-      <c r="D41">
-        <v>4500</v>
-      </c>
-      <c r="E41" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>114</v>
-      </c>
-      <c r="B42" t="s">
-        <v>122</v>
-      </c>
-      <c r="C42" t="s">
-        <v>104</v>
-      </c>
-      <c r="D42">
-        <v>4200</v>
-      </c>
-      <c r="E42" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>114</v>
-      </c>
-      <c r="B43" t="s">
-        <v>123</v>
-      </c>
-      <c r="C43" t="s">
-        <v>124</v>
-      </c>
-      <c r="D43">
-        <v>55000</v>
-      </c>
-      <c r="E43" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>125</v>
-      </c>
-      <c r="B45" t="s">
-        <v>126</v>
-      </c>
-      <c r="C45" t="s">
-        <v>127</v>
-      </c>
-      <c r="D45">
-        <v>8000</v>
-      </c>
-      <c r="E45" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>125</v>
-      </c>
-      <c r="B46" t="s">
-        <v>128</v>
-      </c>
-      <c r="C46" t="s">
-        <v>127</v>
-      </c>
-      <c r="D46">
-        <v>11000</v>
-      </c>
-      <c r="E46" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>125</v>
-      </c>
-      <c r="B47" t="s">
-        <v>129</v>
-      </c>
-      <c r="C47" t="s">
-        <v>127</v>
-      </c>
-      <c r="D47">
-        <v>15000</v>
-      </c>
-      <c r="E47" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>125</v>
-      </c>
-      <c r="B48" t="s">
-        <v>130</v>
-      </c>
-      <c r="C48" t="s">
-        <v>127</v>
-      </c>
-      <c r="D48">
-        <v>19000</v>
-      </c>
-      <c r="E48" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>125</v>
-      </c>
-      <c r="B49" t="s">
-        <v>131</v>
-      </c>
-      <c r="C49" t="s">
-        <v>127</v>
-      </c>
-      <c r="D49">
-        <v>26000</v>
-      </c>
-      <c r="E49" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>125</v>
-      </c>
-      <c r="B50" t="s">
-        <v>132</v>
-      </c>
-      <c r="C50" t="s">
-        <v>124</v>
-      </c>
-      <c r="D50">
-        <v>10000</v>
-      </c>
-      <c r="E50" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>125</v>
-      </c>
-      <c r="B51" t="s">
-        <v>133</v>
-      </c>
-      <c r="C51" t="s">
-        <v>134</v>
-      </c>
-      <c r="D51">
-        <v>1600</v>
-      </c>
-      <c r="E51" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>125</v>
-      </c>
-      <c r="B52" t="s">
-        <v>135</v>
-      </c>
-      <c r="C52" t="s">
-        <v>134</v>
-      </c>
-      <c r="D52">
-        <v>1400</v>
-      </c>
-      <c r="E52" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>125</v>
-      </c>
-      <c r="B53" t="s">
-        <v>136</v>
-      </c>
-      <c r="C53" t="s">
-        <v>134</v>
-      </c>
-      <c r="D53">
-        <v>2000</v>
-      </c>
-      <c r="E53" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>125</v>
-      </c>
-      <c r="B54" t="s">
-        <v>137</v>
-      </c>
-      <c r="C54" t="s">
-        <v>119</v>
-      </c>
-      <c r="D54">
-        <v>8500</v>
-      </c>
-      <c r="E54" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>125</v>
-      </c>
-      <c r="B55" t="s">
-        <v>138</v>
-      </c>
-      <c r="C55" t="s">
-        <v>119</v>
-      </c>
-      <c r="D55">
-        <v>9000</v>
-      </c>
-      <c r="E55" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>125</v>
-      </c>
-      <c r="B56" t="s">
-        <v>139</v>
-      </c>
-      <c r="C56" t="s">
-        <v>119</v>
-      </c>
-      <c r="D56">
-        <v>12000</v>
-      </c>
-      <c r="E56" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>140</v>
-      </c>
-      <c r="B58" t="s">
-        <v>141</v>
-      </c>
-      <c r="C58" t="s">
-        <v>124</v>
-      </c>
-      <c r="D58">
-        <v>32000</v>
-      </c>
-      <c r="E58" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>140</v>
-      </c>
-      <c r="B59" t="s">
-        <v>142</v>
-      </c>
-      <c r="C59" t="s">
-        <v>124</v>
-      </c>
-      <c r="D59">
-        <v>38000</v>
-      </c>
-      <c r="E59" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>140</v>
-      </c>
-      <c r="B60" t="s">
-        <v>143</v>
-      </c>
-      <c r="C60" t="s">
-        <v>124</v>
-      </c>
-      <c r="D60">
-        <v>45000</v>
-      </c>
-      <c r="E60" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>140</v>
-      </c>
-      <c r="B61" t="s">
-        <v>144</v>
-      </c>
-      <c r="C61" t="s">
-        <v>124</v>
-      </c>
-      <c r="D61">
-        <v>30000</v>
-      </c>
-      <c r="E61" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>140</v>
-      </c>
-      <c r="B62" t="s">
-        <v>145</v>
-      </c>
-      <c r="C62" t="s">
-        <v>124</v>
-      </c>
-      <c r="D62">
-        <v>42000</v>
-      </c>
-      <c r="E62" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>146</v>
-      </c>
-      <c r="B64" t="s">
-        <v>147</v>
-      </c>
-      <c r="C64" t="s">
-        <v>119</v>
-      </c>
-      <c r="D64">
-        <v>9000</v>
-      </c>
-      <c r="E64" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>146</v>
-      </c>
-      <c r="B65" t="s">
-        <v>148</v>
-      </c>
-      <c r="C65" t="s">
-        <v>119</v>
-      </c>
-      <c r="D65">
-        <v>8000</v>
-      </c>
-      <c r="E65" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>146</v>
-      </c>
-      <c r="B66" t="s">
-        <v>149</v>
-      </c>
-      <c r="C66" t="s">
-        <v>119</v>
-      </c>
-      <c r="D66">
-        <v>8500</v>
-      </c>
-      <c r="E66" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>146</v>
-      </c>
-      <c r="B67" t="s">
-        <v>150</v>
-      </c>
-      <c r="C67" t="s">
-        <v>104</v>
-      </c>
-      <c r="D67">
-        <v>18000</v>
-      </c>
-      <c r="E67" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>146</v>
-      </c>
-      <c r="B68" t="s">
-        <v>151</v>
-      </c>
-      <c r="C68" t="s">
-        <v>124</v>
-      </c>
-      <c r="D68">
-        <v>15000</v>
-      </c>
-      <c r="E68" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>146</v>
-      </c>
-      <c r="B69" t="s">
-        <v>152</v>
-      </c>
-      <c r="C69" t="s">
-        <v>124</v>
-      </c>
-      <c r="D69">
-        <v>16000</v>
-      </c>
-      <c r="E69" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>146</v>
-      </c>
-      <c r="B70" t="s">
-        <v>153</v>
-      </c>
-      <c r="C70" t="s">
-        <v>124</v>
-      </c>
-      <c r="D70">
-        <v>20000</v>
-      </c>
-      <c r="E70" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>146</v>
-      </c>
-      <c r="B71" t="s">
-        <v>154</v>
-      </c>
-      <c r="C71" t="s">
-        <v>124</v>
-      </c>
-      <c r="D71">
-        <v>22000</v>
-      </c>
-      <c r="E71" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>155</v>
-      </c>
-      <c r="B73" t="s">
-        <v>156</v>
-      </c>
-      <c r="C73" t="s">
-        <v>124</v>
-      </c>
-      <c r="D73">
-        <v>15000</v>
-      </c>
-      <c r="E73" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>155</v>
-      </c>
-      <c r="B74" t="s">
-        <v>157</v>
-      </c>
-      <c r="C74" t="s">
-        <v>124</v>
-      </c>
-      <c r="D74">
-        <v>19000</v>
-      </c>
-      <c r="E74" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>155</v>
-      </c>
-      <c r="B75" t="s">
-        <v>158</v>
-      </c>
-      <c r="C75" t="s">
-        <v>124</v>
-      </c>
-      <c r="D75">
-        <v>12000</v>
-      </c>
-      <c r="E75" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>155</v>
-      </c>
-      <c r="B76" t="s">
-        <v>159</v>
-      </c>
-      <c r="C76" t="s">
-        <v>124</v>
-      </c>
-      <c r="D76">
-        <v>20000</v>
-      </c>
-      <c r="E76" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>155</v>
-      </c>
-      <c r="B77" t="s">
-        <v>160</v>
-      </c>
-      <c r="C77" t="s">
-        <v>161</v>
-      </c>
-      <c r="D77">
-        <v>55000</v>
-      </c>
-      <c r="E77" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>162</v>
-      </c>
-      <c r="B79" t="s">
-        <v>163</v>
-      </c>
-      <c r="C79" t="s">
-        <v>124</v>
-      </c>
-      <c r="D79">
-        <v>22000</v>
-      </c>
-      <c r="E79" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>162</v>
-      </c>
-      <c r="B80" t="s">
-        <v>164</v>
-      </c>
-      <c r="C80" t="s">
-        <v>124</v>
-      </c>
-      <c r="D80">
-        <v>45000</v>
-      </c>
-      <c r="E80" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>162</v>
-      </c>
-      <c r="B81" t="s">
-        <v>165</v>
-      </c>
-      <c r="C81" t="s">
-        <v>124</v>
-      </c>
-      <c r="D81">
-        <v>28000</v>
-      </c>
-      <c r="E81" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>162</v>
-      </c>
-      <c r="B82" t="s">
-        <v>166</v>
-      </c>
-      <c r="C82" t="s">
-        <v>124</v>
-      </c>
-      <c r="D82">
-        <v>60000</v>
-      </c>
-      <c r="E82" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>162</v>
-      </c>
-      <c r="B83" t="s">
-        <v>167</v>
-      </c>
-      <c r="C83" t="s">
-        <v>124</v>
-      </c>
-      <c r="D83">
-        <v>35000</v>
-      </c>
-      <c r="E83" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>168</v>
-      </c>
-      <c r="B85" t="s">
-        <v>169</v>
-      </c>
-      <c r="C85" t="s">
-        <v>170</v>
-      </c>
-      <c r="D85">
-        <v>90000</v>
-      </c>
-      <c r="E85" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>168</v>
-      </c>
-      <c r="B86" t="s">
-        <v>171</v>
-      </c>
-      <c r="C86" t="s">
-        <v>170</v>
-      </c>
-      <c r="D86">
-        <v>110000</v>
-      </c>
-      <c r="E86" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>168</v>
-      </c>
-      <c r="B87" t="s">
-        <v>172</v>
-      </c>
-      <c r="C87" t="s">
-        <v>173</v>
-      </c>
-      <c r="D87">
-        <v>35000</v>
-      </c>
-      <c r="E87" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>168</v>
-      </c>
-      <c r="B88" t="s">
-        <v>174</v>
-      </c>
-      <c r="C88" t="s">
-        <v>173</v>
-      </c>
-      <c r="D88">
-        <v>30000</v>
-      </c>
-      <c r="E88" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>168</v>
-      </c>
-      <c r="B89" t="s">
-        <v>175</v>
-      </c>
-      <c r="C89" t="s">
-        <v>170</v>
-      </c>
-      <c r="D89">
-        <v>120000</v>
-      </c>
-      <c r="E89" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>176</v>
-      </c>
-      <c r="B91" t="s">
-        <v>177</v>
-      </c>
-      <c r="C91" t="s">
-        <v>119</v>
-      </c>
-      <c r="D91">
-        <v>10000</v>
-      </c>
-      <c r="E91" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>176</v>
-      </c>
-      <c r="B92" t="s">
-        <v>178</v>
-      </c>
-      <c r="C92" t="s">
-        <v>119</v>
-      </c>
-      <c r="D92">
-        <v>7000</v>
-      </c>
-      <c r="E92" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>176</v>
-      </c>
-      <c r="B93" t="s">
-        <v>179</v>
-      </c>
-      <c r="C93" t="s">
-        <v>104</v>
-      </c>
-      <c r="D93">
-        <v>2500</v>
-      </c>
-      <c r="E93" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>176</v>
-      </c>
-      <c r="B94" t="s">
-        <v>180</v>
-      </c>
-      <c r="C94" t="s">
-        <v>104</v>
-      </c>
-      <c r="D94">
-        <v>9000</v>
-      </c>
-      <c r="E94" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>176</v>
-      </c>
-      <c r="B95" t="s">
-        <v>181</v>
-      </c>
-      <c r="C95" t="s">
-        <v>104</v>
-      </c>
-      <c r="D95">
-        <v>55000</v>
-      </c>
-      <c r="E95" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>182</v>
-      </c>
-      <c r="B97" t="s">
-        <v>183</v>
-      </c>
-      <c r="C97" t="s">
-        <v>119</v>
-      </c>
-      <c r="D97">
-        <v>1200</v>
-      </c>
-      <c r="E97" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>182</v>
-      </c>
-      <c r="B98" t="s">
-        <v>184</v>
-      </c>
-      <c r="C98" t="s">
-        <v>119</v>
-      </c>
-      <c r="D98">
-        <v>1700</v>
-      </c>
-      <c r="E98" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>182</v>
-      </c>
-      <c r="B99" t="s">
-        <v>185</v>
-      </c>
-      <c r="C99" t="s">
-        <v>119</v>
-      </c>
-      <c r="D99">
-        <v>800</v>
-      </c>
-      <c r="E99" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>182</v>
-      </c>
-      <c r="B100" t="s">
-        <v>186</v>
-      </c>
-      <c r="C100" t="s">
-        <v>104</v>
-      </c>
-      <c r="D100">
-        <v>2000</v>
-      </c>
-      <c r="E100" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>182</v>
-      </c>
-      <c r="B101" t="s">
-        <v>187</v>
-      </c>
-      <c r="C101" t="s">
-        <v>104</v>
-      </c>
-      <c r="D101">
-        <v>35000</v>
-      </c>
-      <c r="E101" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>182</v>
-      </c>
-      <c r="B102" t="s">
-        <v>188</v>
-      </c>
-      <c r="C102" t="s">
-        <v>104</v>
-      </c>
-      <c r="D102">
-        <v>3500</v>
-      </c>
-      <c r="E102" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>182</v>
-      </c>
-      <c r="B103" t="s">
-        <v>189</v>
-      </c>
-      <c r="C103" t="s">
-        <v>104</v>
-      </c>
-      <c r="D103">
-        <v>3200</v>
-      </c>
-      <c r="E103" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
agrego hoja de coca y cocaina
</commit_message>
<xml_diff>
--- a/data/excel.xlsx
+++ b/data/excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abiga\Documents\New project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14148AB6-FD36-460F-888C-845CCB44B34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B04751-224A-48D2-BFE7-BBE420DAE3B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AZUCAR" sheetId="4" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1752" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1763" uniqueCount="439">
   <si>
     <t>Bolsa ingenio</t>
   </si>
@@ -1340,6 +1340,12 @@
   </si>
   <si>
     <t>CLORHIDRATO DE COCAINA</t>
+  </si>
+  <si>
+    <t>estupefaciente</t>
+  </si>
+  <si>
+    <t>planta </t>
   </si>
 </sst>
 </file>
@@ -1350,7 +1356,7 @@
     <numFmt numFmtId="6" formatCode="&quot;$&quot;\ #,##0;[Red]\-&quot;$&quot;\ #,##0"/>
     <numFmt numFmtId="8" formatCode="&quot;$&quot;\ #,##0.00;[Red]\-&quot;$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1386,6 +1392,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1443,7 +1454,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1484,6 +1495,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -4110,10 +4123,65 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15575E2F-B7E9-4EB5-A791-7D7E5CF1065C}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>438</v>
+      </c>
+      <c r="B2" t="s">
+        <v>433</v>
+      </c>
+      <c r="C2" t="s">
+        <v>434</v>
+      </c>
+      <c r="D2">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>437</v>
+      </c>
+      <c r="B3" t="s">
+        <v>436</v>
+      </c>
+      <c r="C3" t="s">
+        <v>435</v>
+      </c>
+      <c r="D3">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="19"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>